<commit_message>
fixed upload logic in backend
</commit_message>
<xml_diff>
--- a/documents/upload-import-excel/mau_import_danh_sach_tai_san_bimlab_updated.xlsx
+++ b/documents/upload-import-excel/mau_import_danh_sach_tai_san_bimlab_updated.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90A72B76-9395-4A0C-BEE4-FCFA2A2C0CAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="HoSoTaiSan_import" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="DanhMuc_ThamChieu" state="visible" r:id="rId5"/>
+    <sheet name="HoSoTaiSan_import" sheetId="1" r:id="rId1"/>
+    <sheet name="DanhMuc_ThamChieu" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase">'HoSoTaiSan_import'!$A$3:$T$3</definedName>
+    <definedName name="_xlnm._FilterDatabase">HoSoTaiSan_import!$A$3:$T$3</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="127">
   <si>
     <t>Không bắt buộc nhập mã tài sản. Nếu để trống, hệ thống sẽ tự sinh theo danh mục node lá.</t>
   </si>
@@ -393,50 +394,56 @@
   </si>
   <si>
     <t>Dịch vụ backup cloud</t>
+  </si>
+  <si>
+    <t>CCDC_TEST</t>
+  </si>
+  <si>
+    <t>Dich vu test</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FF154D7C"/>
-      <sz val="11"/>
       <name val="Be Vietnam Pro"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF64748B"/>
-      <sz val="10"/>
       <name val="Be Vietnam Pro"/>
     </font>
     <font>
       <b/>
+      <sz val="12"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
       <name val="Be Vietnam Pro"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF111827"/>
-      <sz val="11"/>
       <name val="Be Vietnam Pro"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
       <name val="Be Vietnam pro"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
-      <sz val="10"/>
       <name val="Be Vietnam pro"/>
     </font>
   </fonts>
@@ -453,7 +460,7 @@
       </patternFill>
     </fill>
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -543,11 +550,6 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -566,9 +568,14 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -904,12 +911,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T50"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -928,193 +932,193 @@
     <col min="20" max="20" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.95" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:20" ht="33.950000000000003" customHeight="1">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="3"/>
-    </row>
-    <row r="2" ht="24" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8"/>
+      <c r="T1" s="9"/>
+    </row>
+    <row r="2" spans="1:20" ht="24" customHeight="1">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:20" ht="42" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="M3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="N3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="O3" s="5" t="s">
+      <c r="O3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="P3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="Q3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="R3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="S3" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="T3" s="5" t="s">
+      <c r="T3" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6" t="s">
+    <row r="4" spans="1:20" ht="28.5">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="E4" s="6" t="s">
+      <c r="C4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6">
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3">
         <v>28850000</v>
       </c>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6" t="s">
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" ht="28.5">
       <c r="B5" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D5" t="s">
@@ -1130,11 +1134,11 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" ht="28.5">
       <c r="B6" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D6" t="s">
@@ -1150,11 +1154,11 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" ht="28.5">
       <c r="B7" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D7" t="s">
@@ -1170,11 +1174,11 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" ht="28.5">
       <c r="B8" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D8" t="s">
@@ -1190,11 +1194,11 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20">
       <c r="B9" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="3" t="s">
         <v>47</v>
       </c>
       <c r="D9" t="s">
@@ -1210,11 +1214,11 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20">
       <c r="B10" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="3" t="s">
         <v>47</v>
       </c>
       <c r="D10" t="s">
@@ -1230,11 +1234,11 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20">
       <c r="B11" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="3" t="s">
         <v>47</v>
       </c>
       <c r="D11" t="s">
@@ -1250,11 +1254,11 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" ht="28.5">
       <c r="B12" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D12" t="s">
@@ -1270,11 +1274,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" ht="28.5">
       <c r="B13" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D13" t="s">
@@ -1290,11 +1294,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" ht="28.5">
       <c r="B14" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D14" t="s">
@@ -1310,11 +1314,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" ht="28.5">
       <c r="B15" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D15" t="s">
@@ -1330,11 +1334,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" ht="28.5">
       <c r="B16" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D16" t="s">
@@ -1350,11 +1354,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" ht="28.5">
       <c r="B17" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D17" t="s">
@@ -1370,11 +1374,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" ht="28.5">
       <c r="B18" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D18" t="s">
@@ -1390,11 +1394,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" ht="28.5">
       <c r="B19" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D19" t="s">
@@ -1410,11 +1414,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" ht="28.5">
       <c r="B20" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D20" t="s">
@@ -1430,11 +1434,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" ht="28.5">
       <c r="B21" t="s">
         <v>52</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D21" t="s">
@@ -1450,11 +1454,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" ht="28.5">
       <c r="B22" t="s">
         <v>52</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D22" t="s">
@@ -1470,11 +1474,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" ht="28.5">
       <c r="B23" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D23" t="s">
@@ -1490,11 +1494,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:20" ht="28.5">
       <c r="B24" t="s">
         <v>52</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D24" t="s">
@@ -1510,11 +1514,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" ht="28.5">
       <c r="B25" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D25" t="s">
@@ -1530,11 +1534,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" ht="28.5">
       <c r="B26" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D26" t="s">
@@ -1550,11 +1554,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" ht="28.5">
       <c r="B27" t="s">
         <v>52</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D27" t="s">
@@ -1570,11 +1574,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" ht="28.5">
       <c r="B28" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D28" t="s">
@@ -1590,11 +1594,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:20" ht="28.5">
       <c r="B29" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D29" t="s">
@@ -1610,11 +1614,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:20" ht="28.5">
       <c r="B30" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D30" t="s">
@@ -1630,11 +1634,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:20" ht="28.5">
       <c r="B31" t="s">
         <v>55</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D31" t="s">
@@ -1650,11 +1654,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="32" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:20" ht="28.5">
       <c r="B32" t="s">
         <v>55</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D32" t="s">
@@ -1670,11 +1674,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" ht="28.5">
       <c r="B33" t="s">
         <v>55</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D33" t="s">
@@ -1690,11 +1694,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="34" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" ht="28.5">
       <c r="B34" t="s">
         <v>56</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D34" t="s">
@@ -1710,11 +1714,11 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" ht="28.5">
       <c r="B35" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D35" t="s">
@@ -1730,11 +1734,11 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" ht="28.5">
       <c r="B36" t="s">
         <v>60</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D36" t="s">
@@ -1750,45 +1754,45 @@
         <v>62</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A37" s="6"/>
-      <c r="B37" s="6" t="s">
+    <row r="37" spans="1:20" ht="28.5">
+      <c r="A37" s="3"/>
+      <c r="B37" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C37" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D37" s="6" t="s">
+      <c r="C37" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D37" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="E37" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
-      <c r="N37" s="6">
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="3"/>
+      <c r="N37" s="3">
         <v>658400</v>
       </c>
-      <c r="O37" s="6"/>
-      <c r="P37" s="6"/>
-      <c r="Q37" s="6"/>
-      <c r="R37" s="6"/>
-      <c r="S37" s="6"/>
-      <c r="T37" s="6" t="s">
+      <c r="O37" s="3"/>
+      <c r="P37" s="3"/>
+      <c r="Q37" s="3"/>
+      <c r="R37" s="3"/>
+      <c r="S37" s="3"/>
+      <c r="T37" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" ht="28.5">
       <c r="B38" t="s">
         <v>60</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D38" t="s">
@@ -1804,11 +1808,11 @@
         <v>62</v>
       </c>
     </row>
-    <row r="39" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" ht="28.5">
       <c r="B39" t="s">
         <v>60</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D39" t="s">
@@ -1824,11 +1828,11 @@
         <v>62</v>
       </c>
     </row>
-    <row r="40" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" ht="28.5">
       <c r="B40" t="s">
         <v>63</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D40" t="s">
@@ -1844,11 +1848,11 @@
         <v>65</v>
       </c>
     </row>
-    <row r="41" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" ht="28.5">
       <c r="B41" t="s">
         <v>66</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D41" t="s">
@@ -1864,11 +1868,11 @@
         <v>68</v>
       </c>
     </row>
-    <row r="42" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" ht="28.5">
       <c r="B42" t="s">
         <v>69</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D42" t="s">
@@ -1884,11 +1888,11 @@
         <v>71</v>
       </c>
     </row>
-    <row r="43" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" ht="28.5">
       <c r="B43" t="s">
         <v>72</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D43" t="s">
@@ -1904,11 +1908,11 @@
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20">
       <c r="B44" t="s">
         <v>75</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="3" t="s">
         <v>47</v>
       </c>
       <c r="D44" t="s">
@@ -1924,11 +1928,11 @@
         <v>77</v>
       </c>
     </row>
-    <row r="45" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" ht="28.5">
       <c r="B45" t="s">
         <v>78</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D45" t="s">
@@ -1944,11 +1948,11 @@
         <v>80</v>
       </c>
     </row>
-    <row r="46" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20">
       <c r="B46" t="s">
         <v>81</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="3" t="s">
         <v>47</v>
       </c>
       <c r="D46" t="s">
@@ -1964,11 +1968,11 @@
         <v>82</v>
       </c>
     </row>
-    <row r="47" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20">
       <c r="B47" t="s">
         <v>81</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="3" t="s">
         <v>47</v>
       </c>
       <c r="D47" t="s">
@@ -1984,7 +1988,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="48" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20">
       <c r="B48" t="s">
         <v>81</v>
       </c>
@@ -2004,7 +2008,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="49" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:20">
       <c r="B49" t="s">
         <v>83</v>
       </c>
@@ -2024,7 +2028,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="50" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:20">
       <c r="B50" t="s">
         <v>85</v>
       </c>
@@ -2045,66 +2049,33 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:T3"/>
+  <autoFilter ref="A3:T3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:T1"/>
   </mergeCells>
-  <dataValidations count="14">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Sai phân loại" error="Chọn FIXED_ASSET hoặc TOOL_EQUIPMENT." sqref="C100:C200">
+  <dataValidations count="4">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Sai phân loại" error="Chọn FIXED_ASSET hoặc TOOL_EQUIPMENT." sqref="C48:C200" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"FIXED_ASSET,TOOL_EQUIPMENT"</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Sai phân loại" error="Chọn FIXED_ASSET hoặc TOOL_EQUIPMENT." sqref="C48:C200">
-      <formula1>"FIXED_ASSET,TOOL_EQUIPMENT"</formula1>
-    </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Sai phân loại lớp con" error="Chọn một giá trị trong danh sách." sqref="D10:D36">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Sai phân loại lớp con" error="Chọn một giá trị trong danh sách." sqref="D5:D36 D38:D200" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"TANGIBLE,INTANGIBLE,SINGLE_USE,MULTI_USE"</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Sai phân loại lớp con" error="Chọn một giá trị trong danh sách." sqref="D100:D200">
-      <formula1>"TANGIBLE,INTANGIBLE,SINGLE_USE,MULTI_USE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Sai phân loại lớp con" error="Chọn một giá trị trong danh sách." sqref="D38:D200">
-      <formula1>"TANGIBLE,INTANGIBLE,SINGLE_USE,MULTI_USE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Sai phân loại lớp con" error="Chọn một giá trị trong danh sách." sqref="D5:D36">
-      <formula1>"TANGIBLE,INTANGIBLE,SINGLE_USE,MULTI_USE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I10:I36">
+    <dataValidation type="list" allowBlank="1" sqref="I5:I36 I38:I200" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"STRAIGHT_LINE,DECLINING_BALANCE,NONE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I100:I200">
-      <formula1>"STRAIGHT_LINE,DECLINING_BALANCE,NONE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I38:I200">
-      <formula1>"STRAIGHT_LINE,DECLINING_BALANCE,NONE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I5:I36">
-      <formula1>"STRAIGHT_LINE,DECLINING_BALANCE,NONE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="P10:P36">
-      <formula1>"IN_STOCK,ASSIGNED,MAINTENANCE,DISPOSED,LOST,PENDING"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="P100:P200">
-      <formula1>"IN_STOCK,ASSIGNED,MAINTENANCE,DISPOSED,LOST,PENDING"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="P38:P200">
-      <formula1>"IN_STOCK,ASSIGNED,MAINTENANCE,DISPOSED,LOST,PENDING"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="P5:P36">
+    <dataValidation type="list" allowBlank="1" sqref="P5:P36 P38:P200" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"IN_STOCK,ASSIGNED,MAINTENANCE,DISPOSED,LOST,PENDING"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -2112,382 +2083,396 @@
     <col min="4" max="4" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:4" ht="27.95" customHeight="1">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="2" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A2" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D2" s="8"/>
-    </row>
-    <row r="3" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A3" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" s="8" t="s">
+      <c r="B3" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="8"/>
-    </row>
-    <row r="4" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="D3" s="5"/>
+    </row>
+    <row r="4" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A4" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+    <row r="5" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A5" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="6" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A6" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="D6" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A7" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" s="8" t="s">
+      <c r="B7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="D7" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="D7" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A8" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+    <row r="9" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A9" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="10" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+    <row r="10" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A10" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="11" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+    <row r="11" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A11" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="12" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+    <row r="12" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A12" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="13" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+    <row r="13" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A13" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="14" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
+    <row r="14" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A14" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="6" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="15" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
+    <row r="15" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A15" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="16" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+    <row r="16" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A16" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="D16" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A17" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="18" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+    <row r="18" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A18" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="19" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+    <row r="19" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A19" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="20" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+    <row r="20" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A20" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="21" ht="21.95" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
+    <row r="21" spans="1:4" ht="21.95" customHeight="1">
+      <c r="A21" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="D21" s="9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
+      <c r="D21" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="6" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="23" ht="25.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
+    <row r="23" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A23" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="24" ht="25.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+    <row r="24" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A24" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="6" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="25" ht="25.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
+    <row r="25" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A25" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="6" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="26" ht="25.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="8" t="s">
+    <row r="26" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A26" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="6" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="27" ht="25.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="8" t="s">
+    <row r="27" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A27" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="25.5">
+      <c r="A28" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D28" s="6" t="s">
         <v>119</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>